<commit_message>
updated code for frd generation
</commit_message>
<xml_diff>
--- a/backend/test_qrcode_checklist.xlsx
+++ b/backend/test_qrcode_checklist.xlsx
@@ -397,11 +397,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>MX Name: QR Test Merchant</v>
+        <v>MX Name: QR Code Test Merchant</v>
       </c>
       <c r="B1" t="str">
         <v>Audit Checklist</v>
@@ -413,12 +413,12 @@
         <v>Status</v>
       </c>
       <c r="E1" t="str">
-        <v>Comment</v>
+        <v>Comments</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>MID: QR_MID_123</v>
+        <v>MID: QR_MID_999</v>
       </c>
       <c r="B2" t="str">
         <v/>
@@ -438,16 +438,16 @@
         <v/>
       </c>
       <c r="B3" t="str">
-        <v>1. Live Keys</v>
+        <v>Tech Checklist</v>
       </c>
       <c r="C3" t="str">
-        <v/>
+        <v>Configs</v>
       </c>
       <c r="D3" t="str">
-        <v/>
+        <v>Status</v>
       </c>
       <c r="E3" t="str">
-        <v/>
+        <v>Comments</v>
       </c>
     </row>
     <row r="4">
@@ -461,10 +461,10 @@
         <v>Downloading Keys</v>
       </c>
       <c r="D4" t="str">
-        <v>Pass</v>
+        <v>Done</v>
       </c>
       <c r="E4" t="str">
-        <v>Keys downloaded</v>
+        <v>Keys active</v>
       </c>
     </row>
     <row r="5">
@@ -472,16 +472,16 @@
         <v/>
       </c>
       <c r="B5" t="str">
-        <v>2. QR Code Implementation</v>
+        <v/>
       </c>
       <c r="C5" t="str">
-        <v/>
+        <v>Webhook Configs</v>
       </c>
       <c r="D5" t="str">
-        <v/>
+        <v>Done</v>
       </c>
       <c r="E5" t="str">
-        <v/>
+        <v>Integrated</v>
       </c>
     </row>
     <row r="6">
@@ -492,86 +492,18 @@
         <v/>
       </c>
       <c r="C6" t="str">
-        <v>Dashboard</v>
+        <v>Signature Verification</v>
       </c>
       <c r="D6" t="str">
-        <v>Pass</v>
+        <v>Done</v>
       </c>
       <c r="E6" t="str">
-        <v>Dash verified</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v/>
-      </c>
-      <c r="B7" t="str">
-        <v/>
-      </c>
-      <c r="C7" t="str">
-        <v>Instant QR</v>
-      </c>
-      <c r="D7" t="str">
-        <v>N/A</v>
-      </c>
-      <c r="E7" t="str">
-        <v>Not used</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v/>
-      </c>
-      <c r="B8" t="str">
-        <v>Additional Comments</v>
-      </c>
-      <c r="C8" t="str">
-        <v/>
-      </c>
-      <c r="D8" t="str">
-        <v/>
-      </c>
-      <c r="E8" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v/>
-      </c>
-      <c r="B9" t="str">
-        <v>webhook Url for payment</v>
-      </c>
-      <c r="C9" t="str">
-        <v>https://example.com/hook</v>
-      </c>
-      <c r="D9" t="str">
-        <v/>
-      </c>
-      <c r="E9" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v/>
-      </c>
-      <c r="B10" t="str">
-        <v>Webhook Events</v>
-      </c>
-      <c r="C10" t="str">
-        <v>payment.captured, payment.failed</v>
-      </c>
-      <c r="D10" t="str">
-        <v/>
-      </c>
-      <c r="E10" t="str">
-        <v/>
+        <v>Verified</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>